<commit_message>
refactor: update analysis and ETL processes, enhance document handling, and improve notification formatting
</commit_message>
<xml_diff>
--- a/kobo/appeals_monitor_subscription.xlsx
+++ b/kobo/appeals_monitor_subscription.xlsx
@@ -466,7 +466,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -489,7 +488,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -512,7 +510,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -562,7 +559,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -575,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -603,12 +599,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>administration</t>
+          <t>cva</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Administration</t>
+          <t>Cash and Vouchers Assistance (CVA)</t>
         </is>
       </c>
     </row>
@@ -620,12 +616,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>cva</t>
+          <t>communications</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cash and Vouchers Assistance (CVA)</t>
+          <t>Communications</t>
         </is>
       </c>
     </row>
@@ -637,12 +633,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>communications</t>
+          <t>cea</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>Community Engagement and Accountability (CEA)</t>
         </is>
       </c>
     </row>
@@ -654,12 +650,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>cea</t>
+          <t>digital_systems</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Community Engagement and Accountability (CEA)</t>
+          <t>Digital Systems, Tools &amp; Information Technology</t>
         </is>
       </c>
     </row>
@@ -671,12 +667,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>digital_systems</t>
+          <t>green_response</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Digital Systems, Tools &amp; Information Technology</t>
+          <t>Green Response (GR)</t>
         </is>
       </c>
     </row>
@@ -688,12 +684,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>emergency_needs_assessment</t>
+          <t>health</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Emergency Needs Assessment</t>
+          <t>Health</t>
         </is>
       </c>
     </row>
@@ -705,12 +701,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>health</t>
+          <t>humanitarian_diplomacy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Humanitarian Diplomacy</t>
         </is>
       </c>
     </row>
@@ -722,12 +718,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>humanitarian_diplomacy</t>
+          <t>information_management</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Humanitarian Diplomacy</t>
+          <t>Information Management (IM)</t>
         </is>
       </c>
     </row>
@@ -739,12 +735,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>information_management</t>
+          <t>livelihoods</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Information Management (IM)</t>
+          <t>Livelihoods and Basic Needs</t>
         </is>
       </c>
     </row>
@@ -756,12 +752,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>livelihoods</t>
+          <t>logistics</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Livelihoods and Basic Needs</t>
+          <t>Logistics</t>
         </is>
       </c>
     </row>
@@ -773,12 +769,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>logistics</t>
+          <t>migration</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Logistics</t>
+          <t>Migration</t>
         </is>
       </c>
     </row>
@@ -790,12 +786,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>migration</t>
+          <t>operations_management</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Migration</t>
+          <t>Operations Management</t>
         </is>
       </c>
     </row>
@@ -807,12 +803,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>operations_management</t>
+          <t>pmer</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Operations Management</t>
+          <t>Planning, Monitoring, Evaluation and Reporting (PMER)</t>
         </is>
       </c>
     </row>
@@ -824,12 +820,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>pmer</t>
+          <t>pgi</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Planning, Monitoring, Evaluation and Reporting (PMER)</t>
+          <t>Protection, Gender, and Inclusion (PGI)</t>
         </is>
       </c>
     </row>
@@ -841,12 +837,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>pgi</t>
+          <t>relief</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Protection, Gender, and Inclusion (PGI)</t>
+          <t>Relief</t>
         </is>
       </c>
     </row>
@@ -858,12 +854,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>relief</t>
+          <t>security</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Relief</t>
+          <t>Security</t>
         </is>
       </c>
     </row>
@@ -875,12 +871,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>risk_management</t>
+          <t>shelter</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Risk Management</t>
+          <t>Shelter</t>
         </is>
       </c>
     </row>
@@ -892,12 +888,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>security</t>
+          <t>strategic_partnerships</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Strategic Partnerships and Resource Mobilisation</t>
         </is>
       </c>
     </row>
@@ -909,78 +905,44 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>shelter</t>
+          <t>wash</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Shelter</t>
+          <t>Water, Sanitation and Hygiene (WASH)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>sectors</t>
+          <t>yesno</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>strategic_partnerships</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Strategic Partnerships and Resource Mobilisation</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sectors</t>
+          <t>yesno</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>wash</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
-        <is>
-          <t>Water, Sanitation and Hygiene (WASH)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>yesno</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>yesno</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>